<commit_message>
aulas da parte final do semestre
</commit_message>
<xml_diff>
--- a/docs/plano-de-aulas.xlsx
+++ b/docs/plano-de-aulas.xlsx
@@ -88,6 +88,9 @@
     <t xml:space="preserve">implementações + atividades teóricas (ref Feofiloff cap 15)</t>
   </si>
   <si>
+    <t>PI</t>
+  </si>
+  <si>
     <t xml:space="preserve">Intro a Grafos: ADT, componentes e ciclos</t>
   </si>
   <si>
@@ -97,9 +100,6 @@
     <t xml:space="preserve">Definições básicas de grafos: vértices, arestas, grau, ciclos e componentes. (ref Cormen cap 22.1)</t>
   </si>
   <si>
-    <t>PI</t>
-  </si>
-  <si>
     <t xml:space="preserve">Aluno usa ADT matriz ligada para representar grafo e cria alguns grafos manualmente usando a ADT. Aluno cria matrizes de adjacências a partir de um desenho de um grafo (ref Cormen cap 22.1)</t>
   </si>
   <si>
@@ -118,37 +118,37 @@
     <t>BFS</t>
   </si>
   <si>
+    <t xml:space="preserve">BFS + Fila (ref Cormen 22.2)</t>
+  </si>
+  <si>
     <t xml:space="preserve">BFS + Fila (ref Cormen 10.1)</t>
   </si>
   <si>
-    <t xml:space="preserve">BFS + Fila (ref Cormen 22.2)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Grafos com pesos: Dijkstra e caminhos mínimos</t>
   </si>
   <si>
     <t xml:space="preserve">Simulação do algoritmo + implementação da ADT min-heap (ref Cormen 24.3)</t>
   </si>
   <si>
+    <t>PF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Atividades com Ninja para suprir esse gap</t>
+  </si>
+  <si>
+    <t>QUIZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisão Geral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Problemas leetcode para revisão</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avaliação docente + revisão pra prova + montar folha de consulta</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aula de exercícios</t>
-  </si>
-  <si>
-    <t>PF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Atividades com Ninja para suprir esse gap</t>
-  </si>
-  <si>
-    <t>QUIZ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revisão Geral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Problemas leetcode para revisão</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avaliação docente + revisão pra prova + montar folha de consulta</t>
   </si>
   <si>
     <t xml:space="preserve">AULA CANCELADA - LUTO</t>
@@ -425,7 +425,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -465,6 +465,14 @@
     </xf>
     <xf fontId="0" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="center" wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="3" fillId="6" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
@@ -1210,16 +1218,10 @@
         <f t="shared" ref="A12:A28" si="1">A10 + 7</f>
         <v>46097</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>22</v>
-      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="5"/>
       <c r="D12" s="5"/>
-      <c r="E12" s="5" t="s">
-        <v>23</v>
-      </c>
+      <c r="E12" s="5"/>
     </row>
     <row r="13" ht="54.950000000000003" customHeight="1">
       <c r="A13" s="3">
@@ -1227,7 +1229,7 @@
         <v>46101</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
@@ -1258,16 +1260,18 @@
         <f t="shared" si="1"/>
         <v>46111</v>
       </c>
-      <c r="B16" s="4" t="s">
-        <v>21</v>
+      <c r="B16" s="11" t="s">
+        <v>22</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5" t="s">
-        <v>25</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1"/>
     </row>
     <row r="17" ht="36" customHeight="1">
       <c r="A17" s="3">
@@ -1286,15 +1290,15 @@
         <f t="shared" si="1"/>
         <v>46118</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9" t="s">
-        <v>27</v>
+      <c r="B18" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="J18" s="1"/>
     </row>
@@ -1304,14 +1308,14 @@
         <v>46122</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>26</v>
       </c>
       <c r="D19" s="9"/>
       <c r="E19" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J19" s="1"/>
     </row>
@@ -1320,15 +1324,15 @@
         <f t="shared" si="1"/>
         <v>46125</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5" t="s">
-        <v>31</v>
+      <c r="B20" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1">
@@ -1344,7 +1348,7 @@
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1">
@@ -1364,15 +1368,15 @@
         <f t="shared" si="1"/>
         <v>46136</v>
       </c>
-      <c r="B23" s="8" t="s">
+      <c r="B23" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9" t="s">
-        <v>34</v>
+      <c r="C23" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5" t="s">
+        <v>32</v>
       </c>
       <c r="G23" s="7"/>
       <c r="H23" s="1"/>
@@ -1392,7 +1396,7 @@
       </c>
       <c r="D24" s="9"/>
       <c r="E24" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G24" s="7"/>
       <c r="H24" s="1"/>
@@ -1437,7 +1441,7 @@
         <v>46150</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
@@ -1647,7 +1651,7 @@
         <v>20</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
@@ -1671,12 +1675,12 @@
         <f t="shared" si="2"/>
         <v>45912</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
+      <c r="B11" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
       <c r="G11" s="7"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -1688,14 +1692,14 @@
         <v>45915</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" ht="54.950000000000003" customHeight="1">
@@ -1704,7 +1708,7 @@
         <v>45919</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
@@ -1736,14 +1740,14 @@
         <v>45929</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" ht="36" customHeight="1">
@@ -1752,10 +1756,10 @@
         <v>45933</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5" t="s">
@@ -1768,7 +1772,7 @@
         <v>45936</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>26</v>
@@ -1785,7 +1789,7 @@
         <v>45940</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>26</v>
@@ -1809,7 +1813,7 @@
       </c>
       <c r="D20" s="5"/>
       <c r="E20" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1">
@@ -1825,7 +1829,7 @@
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1">
@@ -1833,12 +1837,12 @@
         <f t="shared" si="3"/>
         <v>45950</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
+      <c r="B22" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="3">
@@ -1893,7 +1897,7 @@
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" ht="36" customHeight="1">
@@ -1902,14 +1906,14 @@
         <v>45964</v>
       </c>
       <c r="B26" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="D26" s="5"/>
       <c r="E26" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G26" s="7"/>
       <c r="H26" s="1"/>
@@ -1922,7 +1926,7 @@
         <v>45968</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
@@ -2087,12 +2091,12 @@
         <f>A5+7</f>
         <v>45709</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
       <c r="J7" s="1"/>
     </row>
     <row r="8" ht="36" customHeight="1">
@@ -2100,16 +2104,16 @@
         <f>A6 + 7</f>
         <v>45712</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="15" t="s">
         <v>43</v>
       </c>
       <c r="J8" s="1"/>
@@ -2119,20 +2123,20 @@
         <f>A7 +7</f>
         <v>45716</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="15" t="s">
         <v>43</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
@@ -2140,16 +2144,16 @@
         <f>A8 + 7</f>
         <v>45719</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E10" s="15" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2230,7 +2234,7 @@
         <v>45737</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C15" s="10"/>
       <c r="D15" s="10"/>
@@ -2252,14 +2256,14 @@
         <v>45744</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" ht="36" customHeight="1">
@@ -2268,10 +2272,10 @@
         <v>45747</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="5" t="s">
@@ -2285,7 +2289,7 @@
         <v>45751</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>26</v>
@@ -2302,7 +2306,7 @@
         <v>45754</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>26</v>
@@ -2312,15 +2316,15 @@
         <v>28</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="16" t="s">
         <v>46</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C21" s="9" t="s">
         <v>47</v>
@@ -2343,7 +2347,7 @@
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
@@ -2359,7 +2363,7 @@
       </c>
       <c r="D23" s="5"/>
       <c r="E23" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G23" s="7"/>
       <c r="H23" s="1"/>
@@ -2367,7 +2371,7 @@
       <c r="J23" s="1"/>
     </row>
     <row r="24" ht="36" customHeight="1">
-      <c r="A24" s="14" t="s">
+      <c r="A24" s="16" t="s">
         <v>46</v>
       </c>
       <c r="B24" s="4" t="s">
@@ -2378,7 +2382,7 @@
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="5" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="G24" s="7"/>
       <c r="H24" s="1"/>
@@ -2465,7 +2469,7 @@
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G29" s="7"/>
       <c r="H29" s="1"/>
@@ -2478,17 +2482,17 @@
         <v>45782</v>
       </c>
       <c r="B30" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="D30" s="5"/>
       <c r="E30" s="5" t="s">
         <v>50</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="31" ht="36" customHeight="1">
@@ -2496,17 +2500,17 @@
         <f>A29 +7</f>
         <v>45786</v>
       </c>
-      <c r="B31" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D31" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E31" s="13" t="s">
-        <v>36</v>
+      <c r="B31" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="32" ht="36" customHeight="1">
@@ -2514,17 +2518,17 @@
         <f>A30 + 7</f>
         <v>45789</v>
       </c>
-      <c r="B32" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C32" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D32" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>36</v>
+      <c r="B32" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="33" ht="15"/>
@@ -2588,7 +2592,7 @@
       <c r="E2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2606,7 +2610,7 @@
       <c r="E3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2625,7 +2629,7 @@
       <c r="E4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2644,7 +2648,7 @@
       <c r="E5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2663,7 +2667,7 @@
       <c r="E6" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G6" s="7"/>
@@ -2686,7 +2690,7 @@
       <c r="E7" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G7" s="7"/>
@@ -2709,7 +2713,7 @@
       <c r="E8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G8" s="7"/>
@@ -2732,7 +2736,7 @@
       <c r="E9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2751,7 +2755,7 @@
       <c r="E10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2770,7 +2774,7 @@
       <c r="E11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G11" s="7"/>
@@ -2784,16 +2788,16 @@
         <v>45545</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2803,16 +2807,16 @@
         <v>45548</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="15" t="s">
+      <c r="F13" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2822,14 +2826,14 @@
         <v>45552</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1">
@@ -2837,17 +2841,17 @@
         <f>A13 +7</f>
         <v>45555</v>
       </c>
-      <c r="B15" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>24</v>
+      <c r="B15" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1">
@@ -2855,17 +2859,17 @@
         <f>A14 + 7</f>
         <v>45559</v>
       </c>
-      <c r="B16" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>24</v>
+      <c r="B16" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="17" ht="36" customHeight="1">
@@ -2874,7 +2878,7 @@
         <v>45562</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C17" s="9" t="s">
         <v>26</v>
@@ -2883,7 +2887,7 @@
       <c r="E17" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F17" s="15" t="s">
+      <c r="F17" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2893,7 +2897,7 @@
         <v>45566</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>26</v>
@@ -2902,7 +2906,7 @@
       <c r="E18" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F18" s="15" t="s">
+      <c r="F18" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G18" s="7"/>
@@ -2916,7 +2920,7 @@
         <v>45569</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>47</v>
@@ -2925,7 +2929,7 @@
       <c r="E19" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="F19" s="15" t="s">
+      <c r="F19" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G19" s="7"/>
@@ -2946,9 +2950,9 @@
       </c>
       <c r="D20" s="5"/>
       <c r="E20" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F20" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2965,9 +2969,9 @@
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F21" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="F21" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2980,7 +2984,7 @@
         <v>52</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="5" t="s">
@@ -3006,7 +3010,7 @@
       <c r="E23" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="F23" s="15" t="s">
+      <c r="F23" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3025,7 +3029,7 @@
       <c r="E24" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="F24" s="15" t="s">
+      <c r="F24" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G24" s="7"/>
@@ -3042,7 +3046,7 @@
         <v>52</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D25" s="9"/>
       <c r="E25" s="9" t="s">
@@ -3062,7 +3066,7 @@
         <v>52</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D26" s="9"/>
       <c r="E26" s="9" t="s">
@@ -3079,10 +3083,10 @@
         <v>45597</v>
       </c>
       <c r="B27" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="D27" s="5"/>
       <c r="E27" s="5" t="s">
@@ -3099,10 +3103,10 @@
         <v>45601</v>
       </c>
       <c r="B28" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="D28" s="5"/>
       <c r="E28" s="5" t="s">
@@ -3114,17 +3118,17 @@
         <f>A27 +7</f>
         <v>45604</v>
       </c>
-      <c r="B29" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D29" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>36</v>
+      <c r="B29" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E29" s="15" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="30" ht="36" customHeight="1">
@@ -3132,17 +3136,17 @@
         <f>A28 + 7</f>
         <v>45608</v>
       </c>
-      <c r="B30" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D30" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>36</v>
+      <c r="B30" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -3198,7 +3202,7 @@
       <c r="E2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3216,7 +3220,7 @@
       <c r="E3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3235,7 +3239,7 @@
       <c r="E4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="F4" s="15" t="s">
+      <c r="F4" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3254,7 +3258,7 @@
       <c r="E5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3273,7 +3277,7 @@
       <c r="E6" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G6" s="7"/>
@@ -3296,7 +3300,7 @@
       <c r="E7" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="F7" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G7" s="7"/>
@@ -3319,7 +3323,7 @@
       <c r="E8" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="15" t="s">
+      <c r="F8" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G8" s="7"/>
@@ -3342,7 +3346,7 @@
       <c r="E9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="15" t="s">
+      <c r="F9" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3361,7 +3365,7 @@
       <c r="E10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F10" s="15" t="s">
+      <c r="F10" s="17" t="s">
         <v>51</v>
       </c>
     </row>
@@ -3380,7 +3384,7 @@
       <c r="E11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F11" s="15" t="s">
+      <c r="F11" s="17" t="s">
         <v>51</v>
       </c>
       <c r="G11" s="7"/>
@@ -3394,16 +3398,16 @@
         <v>45545</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="19" t="s">
         <v>55</v>
       </c>
     </row>
@@ -3413,16 +3417,16 @@
         <v>45548</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="19" t="s">
         <v>55</v>
       </c>
     </row>
@@ -3432,14 +3436,14 @@
         <v>45552</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1">
@@ -3447,17 +3451,17 @@
         <f>A13 +7</f>
         <v>45555</v>
       </c>
-      <c r="B15" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>24</v>
+      <c r="B15" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1">
@@ -3465,17 +3469,17 @@
         <f>A14 + 7</f>
         <v>45559</v>
       </c>
-      <c r="B16" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>24</v>
+      <c r="B16" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="17" ht="36" customHeight="1">
@@ -3483,15 +3487,15 @@
         <f>A15 +7</f>
         <v>45562</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="B17" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="19" t="s">
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="19" t="s">
         <v>55</v>
       </c>
     </row>
@@ -3501,7 +3505,7 @@
         <v>45566</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>26</v>
@@ -3510,7 +3514,7 @@
       <c r="E18" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F18" s="20" t="s">
+      <c r="F18" s="22" t="s">
         <v>58</v>
       </c>
       <c r="G18" s="7"/>
@@ -3524,7 +3528,7 @@
         <v>45569</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C19" s="9" t="s">
         <v>26</v>
@@ -3533,7 +3537,7 @@
       <c r="E19" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="F19" s="20" t="s">
+      <c r="F19" s="22" t="s">
         <v>58</v>
       </c>
       <c r="G19" s="7"/>
@@ -3547,7 +3551,7 @@
         <v>45573</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>47</v>
@@ -3570,9 +3574,9 @@
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F21" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" s="22" t="s">
         <v>58</v>
       </c>
     </row>
@@ -3589,9 +3593,9 @@
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="F22" s="22" t="s">
         <v>58</v>
       </c>
       <c r="G22" s="7"/>
@@ -3608,7 +3612,7 @@
         <v>52</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D23" s="5"/>
       <c r="E23" s="5" t="s">
@@ -3630,7 +3634,7 @@
       <c r="E24" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="F24" s="20" t="s">
+      <c r="F24" s="22" t="s">
         <v>58</v>
       </c>
       <c r="G24" s="7"/>
@@ -3653,7 +3657,7 @@
       <c r="E25" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="F25" s="20" t="s">
+      <c r="F25" s="22" t="s">
         <v>58</v>
       </c>
       <c r="G25" s="7"/>
@@ -3670,7 +3674,7 @@
         <v>52</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D26" s="9"/>
       <c r="E26" s="9" t="s">
@@ -3690,7 +3694,7 @@
         <v>52</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D27" s="9"/>
       <c r="E27" s="9" t="s">
@@ -3707,10 +3711,10 @@
         <v>45601</v>
       </c>
       <c r="B28" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="D28" s="5"/>
       <c r="E28" s="5" t="s">
@@ -3722,17 +3726,17 @@
         <f>A27 +7</f>
         <v>45604</v>
       </c>
-      <c r="B29" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D29" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E29" s="13" t="s">
-        <v>36</v>
+      <c r="B29" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E29" s="15" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="30" ht="36" customHeight="1">
@@ -3740,17 +3744,17 @@
         <f>A28 + 7</f>
         <v>45608</v>
       </c>
-      <c r="B30" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="D30" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="E30" s="13" t="s">
-        <v>36</v>
+      <c r="B30" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -3776,16 +3780,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="15">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="23" t="s">
         <v>3</v>
       </c>
     </row>
@@ -3793,13 +3797,13 @@
       <c r="A2" s="7">
         <v>45327</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="23" t="s">
         <v>59</v>
       </c>
     </row>
@@ -3807,44 +3811,44 @@
       <c r="A3" s="7">
         <v>45331</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="E3" s="23" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="4" ht="15">
-      <c r="A4" s="23">
+      <c r="A4" s="25">
         <f>A2 + 7</f>
         <v>45334</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="B4" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="E4" s="25"/>
+      <c r="E4" s="27"/>
     </row>
     <row r="5" ht="41.75">
       <c r="A5" s="7">
         <f>A3 +7</f>
         <v>45338</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="23" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="21" t="s">
+      <c r="E5" s="23" t="s">
         <v>62</v>
       </c>
     </row>
@@ -3853,13 +3857,13 @@
         <f>A4 + 7</f>
         <v>45341</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="23" t="s">
         <v>63</v>
       </c>
     </row>
@@ -3868,13 +3872,13 @@
         <f>A5 +7</f>
         <v>45345</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="21" t="s">
+      <c r="C7" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="23" t="s">
         <v>64</v>
       </c>
     </row>
@@ -3883,13 +3887,13 @@
         <f>A6 + 7</f>
         <v>45348</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="21" t="s">
+      <c r="E8" s="23" t="s">
         <v>63</v>
       </c>
     </row>
@@ -3898,13 +3902,13 @@
         <f>A7 +7</f>
         <v>45352</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" s="21" t="s">
+      <c r="C9" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="23" t="s">
         <v>63</v>
       </c>
     </row>
@@ -3913,13 +3917,13 @@
         <f>A8 + 7</f>
         <v>45355</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="E10" s="21" t="s">
+      <c r="E10" s="23" t="s">
         <v>63</v>
       </c>
     </row>
@@ -3928,13 +3932,13 @@
         <f>A9 +7</f>
         <v>45359</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" s="21" t="s">
+      <c r="C11" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="23" t="s">
         <v>63</v>
       </c>
     </row>
@@ -3943,13 +3947,13 @@
         <f>A10 + 7</f>
         <v>45362</v>
       </c>
-      <c r="B12" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="C12" s="21" t="s">
+      <c r="B12" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="21" t="s">
+      <c r="C12" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="23" t="s">
         <v>66</v>
       </c>
     </row>
@@ -3958,13 +3962,13 @@
         <f>A11 +7</f>
         <v>45366</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E13" s="21" t="s">
+      <c r="C13" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="23" t="s">
         <v>64</v>
       </c>
     </row>
@@ -3973,13 +3977,13 @@
         <f>A12 + 7</f>
         <v>45369</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="E14" s="23" t="s">
         <v>68</v>
       </c>
     </row>
@@ -3988,17 +3992,17 @@
         <f>A13 +7</f>
         <v>45373</v>
       </c>
-      <c r="B15" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="C15" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15" s="26" t="s">
-        <v>24</v>
+      <c r="B15" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" s="28" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="16" ht="40.25" customHeight="1">
@@ -4006,34 +4010,34 @@
         <f>A14 + 7</f>
         <v>45376</v>
       </c>
-      <c r="B16" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="C16" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="E16" s="26" t="s">
-        <v>24</v>
+      <c r="B16" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="D16" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="28" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="17" ht="15">
-      <c r="A17" s="23">
+      <c r="A17" s="25">
         <f>A15 +7</f>
         <v>45380</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="26" t="s">
+      <c r="C17" s="28" t="s">
         <v>61</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="E17" s="24" t="s">
+      <c r="E17" s="26" t="s">
         <v>61</v>
       </c>
       <c r="I17" s="7"/>
@@ -4043,13 +4047,13 @@
         <f>A16 + 7</f>
         <v>45383</v>
       </c>
-      <c r="B18" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="21" t="s">
+      <c r="B18" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="E18" s="21" t="s">
+      <c r="C18" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" s="23" t="s">
         <v>66</v>
       </c>
     </row>
@@ -4058,13 +4062,13 @@
         <f>A17 +7</f>
         <v>45387</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E19" s="21" t="s">
+      <c r="C19" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E19" s="23" t="s">
         <v>64</v>
       </c>
       <c r="I19" s="7"/>
@@ -4074,13 +4078,13 @@
         <f>A18 + 7</f>
         <v>45390</v>
       </c>
-      <c r="B20" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="21" t="s">
+      <c r="B20" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="21" t="s">
+      <c r="E20" s="23" t="s">
         <v>69</v>
       </c>
     </row>
@@ -4089,13 +4093,13 @@
         <f>A19 +7</f>
         <v>45394</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="C21" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E21" s="21" t="s">
+      <c r="C21" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E21" s="23" t="s">
         <v>64</v>
       </c>
     </row>
@@ -4104,13 +4108,13 @@
         <f>A20 + 7</f>
         <v>45397</v>
       </c>
-      <c r="B22" s="22" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="21" t="s">
+      <c r="B22" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="E22" s="21" t="s">
+      <c r="E22" s="23" t="s">
         <v>70</v>
       </c>
     </row>
@@ -4119,13 +4123,13 @@
         <f>A21 +7</f>
         <v>45401</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="C23" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E23" s="21" t="s">
+      <c r="C23" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E23" s="23" t="s">
         <v>64</v>
       </c>
     </row>
@@ -4134,13 +4138,13 @@
         <f>A22 + 7</f>
         <v>45404</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C24" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="E24" s="21" t="s">
+      <c r="E24" s="23" t="s">
         <v>71</v>
       </c>
       <c r="I24" s="7"/>
@@ -4150,13 +4154,13 @@
         <f>A23 +7</f>
         <v>45408</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E25" s="21" t="s">
+      <c r="C25" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E25" s="23" t="s">
         <v>64</v>
       </c>
     </row>
@@ -4165,13 +4169,13 @@
         <f>A24 + 7</f>
         <v>45411</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="E26" s="21" t="s">
+      <c r="E26" s="23" t="s">
         <v>72</v>
       </c>
     </row>
@@ -4180,13 +4184,13 @@
         <f>A25 +7</f>
         <v>45415</v>
       </c>
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="C27" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E27" s="21" t="s">
+      <c r="C27" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E27" s="23" t="s">
         <v>64</v>
       </c>
     </row>
@@ -4195,50 +4199,50 @@
         <f>A26 + 7</f>
         <v>45418</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="C28" s="21" t="s">
-        <v>40</v>
-      </c>
-      <c r="E28" s="21" t="s">
+      <c r="C28" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="E28" s="23" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="29" ht="15">
-      <c r="A29" s="23">
+      <c r="A29" s="25">
         <f>A27 +7</f>
         <v>45422</v>
       </c>
-      <c r="B29" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="D29" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="E29" s="26" t="s">
-        <v>36</v>
+      <c r="B29" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="D29" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="E29" s="28" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="30" ht="15">
-      <c r="A30" s="23">
+      <c r="A30" s="25">
         <f>A28 + 7</f>
         <v>45425</v>
       </c>
-      <c r="B30" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="D30" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="E30" s="26" t="s">
-        <v>36</v>
+      <c r="B30" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="D30" s="28" t="s">
+        <v>35</v>
+      </c>
+      <c r="E30" s="28" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -4270,18 +4274,18 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="23" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" ht="15">
-      <c r="A2" s="27">
+      <c r="A2" s="29">
         <v>45152</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="29" t="s">
         <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -4289,22 +4293,22 @@
       </c>
     </row>
     <row r="3" ht="15">
-      <c r="A3" s="27">
+      <c r="A3" s="29">
         <v>45156</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="B3" s="29" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" s="25" customFormat="1" ht="15">
-      <c r="A4" s="27">
+    <row r="4" s="27" customFormat="1" ht="15">
+      <c r="A4" s="29">
         <f>A2 + 7</f>
         <v>45159</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="29" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -4317,11 +4321,11 @@
       <c r="H4" s="1"/>
     </row>
     <row r="5" ht="15">
-      <c r="A5" s="27">
+      <c r="A5" s="29">
         <f>A3 +7</f>
         <v>45163</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="29" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -4332,27 +4336,27 @@
       </c>
     </row>
     <row r="6" ht="15">
-      <c r="A6" s="27">
+      <c r="A6" s="29">
         <f>A4 + 7</f>
         <v>45166</v>
       </c>
-      <c r="B6" s="27" t="s">
-        <v>21</v>
+      <c r="B6" s="29" t="s">
+        <v>22</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="7" ht="15">
-      <c r="A7" s="27">
+      <c r="A7" s="29">
         <f>A5 +7</f>
         <v>45170</v>
       </c>
-      <c r="B7" s="27" t="s">
-        <v>21</v>
+      <c r="B7" s="29" t="s">
+        <v>22</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>26</v>
@@ -4362,12 +4366,12 @@
       </c>
     </row>
     <row r="8" ht="15">
-      <c r="A8" s="27">
+      <c r="A8" s="29">
         <f>A6 + 7</f>
         <v>45173</v>
       </c>
-      <c r="B8" s="27" t="s">
-        <v>21</v>
+      <c r="B8" s="29" t="s">
+        <v>22</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>47</v>
@@ -4380,19 +4384,19 @@
       <c r="H8" s="1"/>
     </row>
     <row r="9" ht="15">
-      <c r="A9" s="23">
+      <c r="A9" s="25">
         <f>A7 +7</f>
         <v>45177</v>
       </c>
-      <c r="B9" s="23"/>
-      <c r="C9" s="25" t="s">
+      <c r="B9" s="25"/>
+      <c r="C9" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="D9" s="25"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="25"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
     </row>
     <row r="10" ht="15">
       <c r="A10" s="7">
@@ -4429,10 +4433,10 @@
         <f>A10 + 7</f>
         <v>45187</v>
       </c>
-      <c r="B12" s="28" t="s">
+      <c r="B12" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="19" t="s">
         <v>73</v>
       </c>
     </row>
@@ -4441,9 +4445,9 @@
         <f>A11 +7</f>
         <v>45191</v>
       </c>
-      <c r="B13" s="29"/>
-      <c r="C13" s="30" t="s">
-        <v>24</v>
+      <c r="B13" s="31"/>
+      <c r="C13" s="32" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="14" ht="15">
@@ -4451,9 +4455,9 @@
         <f>A12 + 7</f>
         <v>45194</v>
       </c>
-      <c r="B14" s="29"/>
-      <c r="C14" s="30" t="s">
-        <v>24</v>
+      <c r="B14" s="31"/>
+      <c r="C14" s="32" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="15" ht="15">
@@ -4479,10 +4483,10 @@
         <f>A14 + 7</f>
         <v>45201</v>
       </c>
-      <c r="B16" s="28" t="s">
+      <c r="B16" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="19" t="s">
         <v>77</v>
       </c>
     </row>
@@ -4511,19 +4515,19 @@
       </c>
     </row>
     <row r="19" ht="15">
-      <c r="A19" s="23">
+      <c r="A19" s="25">
         <f>A17 +7</f>
         <v>45212</v>
       </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="25" t="s">
+      <c r="B19" s="25"/>
+      <c r="C19" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="27"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="27"/>
     </row>
     <row r="20" ht="15">
       <c r="A20" s="7">
@@ -4589,19 +4593,19 @@
       </c>
     </row>
     <row r="25" ht="15">
-      <c r="A25" s="23">
+      <c r="A25" s="25">
         <f>A23 +7</f>
         <v>45233</v>
       </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="25" t="s">
+      <c r="B25" s="25"/>
+      <c r="C25" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="27"/>
+      <c r="H25" s="27"/>
     </row>
     <row r="26" ht="15">
       <c r="A26" s="7">
@@ -4616,13 +4620,13 @@
       </c>
     </row>
     <row r="27" ht="15">
-      <c r="A27" s="29">
+      <c r="A27" s="31">
         <f>A25 +7</f>
         <v>45240</v>
       </c>
-      <c r="B27" s="29"/>
-      <c r="C27" s="30" t="s">
-        <v>36</v>
+      <c r="B27" s="31"/>
+      <c r="C27" s="32" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="30" ht="15">

</xml_diff>